<commit_message>
Add NAIRU estimation pipeline and data
Introduce a new NAIRU estimation workflow: add src/nairu package (estimation and model core) and pipeline scripts (build_nairu_dataset, run_nairu_estimation). Add input datasets (Data_NAIRU.xlsx, PIB_CO.xlsx, icu_historical.csv and a temporary ~$PIB_CO.xlsx) and documentation (docs/NAIRU_estimation_process.pdf). Update processed data files (expanded andi_capacidad_instalada.csv with full historical series and modify dane_gdp_colombia.csv and viog_colombia.csv) and adjust src/main.py and source connectors (EOIC/DANE/ViOG) to integrate the new pipeline and data.
</commit_message>
<xml_diff>
--- a/data/inputs/PIB_CO.xlsx
+++ b/data/inputs/PIB_CO.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D118"/>
+  <dimension ref="A1:D129"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2086,6 +2086,160 @@
         <v>0.006265344387101246</v>
       </c>
     </row>
+    <row r="119">
+      <c r="A119" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B119" t="n">
+        <v>2</v>
+      </c>
+      <c r="C119" t="n">
+        <v>244468.8669</v>
+      </c>
+      <c r="D119" t="n">
+        <v>-0.006295724380417256</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B120" t="n">
+        <v>3</v>
+      </c>
+      <c r="C120" t="n">
+        <v>244178.5966</v>
+      </c>
+      <c r="D120" t="n">
+        <v>-0.00118735078082044</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B121" t="n">
+        <v>4</v>
+      </c>
+      <c r="C121" t="n">
+        <v>246177.8098</v>
+      </c>
+      <c r="D121" t="n">
+        <v>0.008187503851023514</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B122" t="n">
+        <v>1</v>
+      </c>
+      <c r="C122" t="n">
+        <v>246721.9338</v>
+      </c>
+      <c r="D122" t="n">
+        <v>0.002210288573296193</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B123" t="n">
+        <v>2</v>
+      </c>
+      <c r="C123" t="n">
+        <v>248617.8079</v>
+      </c>
+      <c r="D123" t="n">
+        <v>0.007684254378197641</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B124" t="n">
+        <v>3</v>
+      </c>
+      <c r="C124" t="n">
+        <v>248237.3609</v>
+      </c>
+      <c r="D124" t="n">
+        <v>-0.001530248388937006</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B125" t="n">
+        <v>4</v>
+      </c>
+      <c r="C125" t="n">
+        <v>251912.8973</v>
+      </c>
+      <c r="D125" t="n">
+        <v>0.01480653994497083</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B126" t="n">
+        <v>1</v>
+      </c>
+      <c r="C126" t="n">
+        <v>253089.4119</v>
+      </c>
+      <c r="D126" t="n">
+        <v>0.00467032300691983</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B127" t="n">
+        <v>2</v>
+      </c>
+      <c r="C127" t="n">
+        <v>253990.2704</v>
+      </c>
+      <c r="D127" t="n">
+        <v>0.003559447600897547</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B128" t="n">
+        <v>3</v>
+      </c>
+      <c r="C128" t="n">
+        <v>257201.0399</v>
+      </c>
+      <c r="D128" t="n">
+        <v>0.01264130903496219</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B129" t="n">
+        <v>4</v>
+      </c>
+      <c r="C129" t="n">
+        <v>257510.2116</v>
+      </c>
+      <c r="D129" t="n">
+        <v>0.001202062402703374</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: regenerar VIOG con Kalman corregido
</commit_message>
<xml_diff>
--- a/data/inputs/PIB_CO.xlsx
+++ b/data/inputs/PIB_CO.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D129"/>
+  <dimension ref="A1:D130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -458,7 +458,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>96060.8250015524</v>
+        <v>96061.14977942497</v>
       </c>
       <c r="D2" t="inlineStr"/>
     </row>
@@ -470,10 +470,10 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>97730.65726621717</v>
+        <v>97730.98768972697</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01738307228402203</v>
+        <v>0.01738307228402181</v>
       </c>
     </row>
     <row r="4">
@@ -484,7 +484,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>99703.62336226639</v>
+        <v>99703.96045629699</v>
       </c>
       <c r="D4" t="n">
         <v>0.02018779113164948</v>
@@ -498,7 +498,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>100058.8325520385</v>
+        <v>100059.1708470174</v>
       </c>
       <c r="D5" t="n">
         <v>0.003562650762264585</v>
@@ -512,10 +512,10 @@
         <v>1</v>
       </c>
       <c r="C6" t="n">
-        <v>101996.1104772321</v>
+        <v>101996.4553220715</v>
       </c>
       <c r="D6" t="n">
-        <v>0.01936138845299884</v>
+        <v>0.01936138845299862</v>
       </c>
     </row>
     <row r="7">
@@ -526,7 +526,7 @@
         <v>2</v>
       </c>
       <c r="C7" t="n">
-        <v>103154.8221669072</v>
+        <v>103155.1709293053</v>
       </c>
       <c r="D7" t="n">
         <v>0.01136035172570415</v>
@@ -540,7 +540,7 @@
         <v>3</v>
       </c>
       <c r="C8" t="n">
-        <v>103584.2807010411</v>
+        <v>103584.6309154216</v>
       </c>
       <c r="D8" t="n">
         <v>0.004163242445797355</v>
@@ -554,7 +554,7 @@
         <v>4</v>
       </c>
       <c r="C9" t="n">
-        <v>105293.122863764</v>
+        <v>105293.4788556727</v>
       </c>
       <c r="D9" t="n">
         <v>0.01649711858940095</v>
@@ -568,7 +568,7 @@
         <v>1</v>
       </c>
       <c r="C10" t="n">
-        <v>105029.3485859326</v>
+        <v>105029.7036860308</v>
       </c>
       <c r="D10" t="n">
         <v>-0.002505142507480351</v>
@@ -582,7 +582,7 @@
         <v>2</v>
       </c>
       <c r="C11" t="n">
-        <v>105489.1805273983</v>
+        <v>105489.5371821702</v>
       </c>
       <c r="D11" t="n">
         <v>0.004378128091401701</v>
@@ -596,7 +596,7 @@
         <v>3</v>
       </c>
       <c r="C12" t="n">
-        <v>105866.8026343995</v>
+        <v>105867.1605658969</v>
       </c>
       <c r="D12" t="n">
         <v>0.003579723580307004</v>
@@ -610,7 +610,7 @@
         <v>4</v>
       </c>
       <c r="C13" t="n">
-        <v>106154.8255208087</v>
+        <v>106155.1844261001</v>
       </c>
       <c r="D13" t="n">
         <v>0.002720615709948415</v>
@@ -624,7 +624,7 @@
         <v>1</v>
       </c>
       <c r="C14" t="n">
-        <v>105865.5555298007</v>
+        <v>105865.9134570817</v>
       </c>
       <c r="D14" t="n">
         <v>-0.002724982021201305</v>
@@ -638,7 +638,7 @@
         <v>2</v>
       </c>
       <c r="C15" t="n">
-        <v>109488.6333205971</v>
+        <v>109489.0034973616</v>
       </c>
       <c r="D15" t="n">
         <v>0.03422338618698784</v>
@@ -652,7 +652,7 @@
         <v>3</v>
       </c>
       <c r="C16" t="n">
-        <v>110344.5550067912</v>
+        <v>110344.9280773933</v>
       </c>
       <c r="D16" t="n">
         <v>0.00781744789605554</v>
@@ -666,7 +666,7 @@
         <v>4</v>
       </c>
       <c r="C17" t="n">
-        <v>111335.7817143645</v>
+        <v>111336.1581362652</v>
       </c>
       <c r="D17" t="n">
         <v>0.008983014227682995</v>
@@ -680,7 +680,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="n">
-        <v>111828.4812723596</v>
+        <v>111828.8593600581</v>
       </c>
       <c r="D18" t="n">
         <v>0.004425347811892966</v>
@@ -694,10 +694,10 @@
         <v>2</v>
       </c>
       <c r="C19" t="n">
-        <v>111930.1319523457</v>
+        <v>111930.5103837212</v>
       </c>
       <c r="D19" t="n">
-        <v>0.0009089873959620132</v>
+        <v>0.0009089873959617911</v>
       </c>
     </row>
     <row r="20">
@@ -708,7 +708,7 @@
         <v>3</v>
       </c>
       <c r="C20" t="n">
-        <v>109303.1410805031</v>
+        <v>109303.5106301257</v>
       </c>
       <c r="D20" t="n">
         <v>-0.02346991668839493</v>
@@ -722,10 +722,10 @@
         <v>4</v>
       </c>
       <c r="C21" t="n">
-        <v>106462.924460222</v>
+        <v>106463.2844071839</v>
       </c>
       <c r="D21" t="n">
-        <v>-0.02598476669750283</v>
+        <v>-0.02598476669750271</v>
       </c>
     </row>
     <row r="22">
@@ -736,7 +736,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="n">
-        <v>105214.8816191677</v>
+        <v>105215.2373465458</v>
       </c>
       <c r="D22" t="n">
         <v>-0.01172279314495683</v>
@@ -750,7 +750,7 @@
         <v>2</v>
       </c>
       <c r="C23" t="n">
-        <v>104297.4671865874</v>
+        <v>104297.8198122234</v>
       </c>
       <c r="D23" t="n">
         <v>-0.008719436057542773</v>
@@ -764,7 +764,7 @@
         <v>3</v>
       </c>
       <c r="C24" t="n">
-        <v>105818.2180033702</v>
+        <v>105818.5757706049</v>
       </c>
       <c r="D24" t="n">
         <v>0.01458089882530111</v>
@@ -778,10 +778,10 @@
         <v>4</v>
       </c>
       <c r="C25" t="n">
-        <v>105716.4274611861</v>
+        <v>105716.7848842709</v>
       </c>
       <c r="D25" t="n">
-        <v>-0.0009619377844832799</v>
+        <v>-0.000961937784483391</v>
       </c>
     </row>
     <row r="26">
@@ -792,10 +792,10 @@
         <v>1</v>
       </c>
       <c r="C26" t="n">
-        <v>107101.4974938672</v>
+        <v>107101.8347873777</v>
       </c>
       <c r="D26" t="n">
-        <v>0.01310174838427725</v>
+        <v>0.01310151367753987</v>
       </c>
     </row>
     <row r="27">
@@ -806,7 +806,7 @@
         <v>2</v>
       </c>
       <c r="C27" t="n">
-        <v>107160.4042237462</v>
+        <v>107160.741702771</v>
       </c>
       <c r="D27" t="n">
         <v>0.0005500084616685275</v>
@@ -820,10 +820,10 @@
         <v>3</v>
       </c>
       <c r="C28" t="n">
-        <v>107918.6395673171</v>
+        <v>107918.9794342437</v>
       </c>
       <c r="D28" t="n">
-        <v>0.00707570439905858</v>
+        <v>0.007075704399058358</v>
       </c>
     </row>
     <row r="29">
@@ -834,10 +834,10 @@
         <v>4</v>
       </c>
       <c r="C29" t="n">
-        <v>107930.7229990871</v>
+        <v>107931.062904068</v>
       </c>
       <c r="D29" t="n">
-        <v>0.0001119679771584003</v>
+        <v>0.0001119679771586224</v>
       </c>
     </row>
     <row r="30">
@@ -848,7 +848,7 @@
         <v>1</v>
       </c>
       <c r="C30" t="n">
-        <v>108471.456570797</v>
+        <v>108471.7981787038</v>
       </c>
       <c r="D30" t="n">
         <v>0.00501000601760504</v>
@@ -862,7 +862,7 @@
         <v>2</v>
       </c>
       <c r="C31" t="n">
-        <v>108630.051612779</v>
+        <v>108630.3937201473</v>
       </c>
       <c r="D31" t="n">
         <v>0.001462090092599011</v>
@@ -876,7 +876,7 @@
         <v>3</v>
       </c>
       <c r="C32" t="n">
-        <v>109676.7788898598</v>
+        <v>109677.1242936743</v>
       </c>
       <c r="D32" t="n">
         <v>0.009635706340378247</v>
@@ -890,10 +890,10 @@
         <v>4</v>
       </c>
       <c r="C33" t="n">
-        <v>110549.8068352462</v>
+        <v>110550.1549884775</v>
       </c>
       <c r="D33" t="n">
-        <v>0.007960007161252003</v>
+        <v>0.007960007161252225</v>
       </c>
     </row>
     <row r="34">
@@ -904,10 +904,10 @@
         <v>1</v>
       </c>
       <c r="C34" t="n">
-        <v>109420.0059647462</v>
+        <v>109420.3505599087</v>
       </c>
       <c r="D34" t="n">
-        <v>-0.01021983577215779</v>
+        <v>-0.0102198357721579</v>
       </c>
     </row>
     <row r="35">
@@ -918,7 +918,7 @@
         <v>2</v>
       </c>
       <c r="C35" t="n">
-        <v>113055.608498561</v>
+        <v>113055.9645432846</v>
       </c>
       <c r="D35" t="n">
         <v>0.03322612260673918</v>
@@ -932,10 +932,10 @@
         <v>3</v>
       </c>
       <c r="C36" t="n">
-        <v>112830.5545818437</v>
+        <v>112830.9099178076</v>
       </c>
       <c r="D36" t="n">
-        <v>-0.001990647962591852</v>
+        <v>-0.001990647962591963</v>
       </c>
     </row>
     <row r="37">
@@ -946,7 +946,7 @@
         <v>4</v>
       </c>
       <c r="C37" t="n">
-        <v>112972.5349051419</v>
+        <v>112972.8906882428</v>
       </c>
       <c r="D37" t="n">
         <v>0.001258349955154614</v>
@@ -960,7 +960,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="n">
-        <v>113860.6671402408</v>
+        <v>113861.0257203263</v>
       </c>
       <c r="D38" t="n">
         <v>0.007861488067384181</v>
@@ -974,7 +974,7 @@
         <v>2</v>
       </c>
       <c r="C39" t="n">
-        <v>115861.9855271558</v>
+        <v>115862.3504099703</v>
       </c>
       <c r="D39" t="n">
         <v>0.01757690726025762</v>
@@ -988,10 +988,10 @@
         <v>3</v>
       </c>
       <c r="C40" t="n">
-        <v>117302.9347657347</v>
+        <v>117303.3041865139</v>
       </c>
       <c r="D40" t="n">
-        <v>0.01243677321791714</v>
+        <v>0.01243677321791736</v>
       </c>
     </row>
     <row r="41">
@@ -1002,7 +1002,7 @@
         <v>4</v>
       </c>
       <c r="C41" t="n">
-        <v>118817.8950239051</v>
+        <v>118818.2692157312</v>
       </c>
       <c r="D41" t="n">
         <v>0.01291493909505292</v>
@@ -1016,7 +1016,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="n">
-        <v>121020.1004639973</v>
+        <v>121020.4815912036</v>
       </c>
       <c r="D42" t="n">
         <v>0.01853429098074111</v>
@@ -1030,10 +1030,10 @@
         <v>2</v>
       </c>
       <c r="C43" t="n">
-        <v>120946.0894444058</v>
+        <v>120946.47033853</v>
       </c>
       <c r="D43" t="n">
-        <v>-0.0006115597269198414</v>
+        <v>-0.0006115597269199524</v>
       </c>
     </row>
     <row r="44">
@@ -1044,7 +1044,7 @@
         <v>3</v>
       </c>
       <c r="C44" t="n">
-        <v>122359.850961502</v>
+        <v>122360.2363079691</v>
       </c>
       <c r="D44" t="n">
         <v>0.011689187501561</v>
@@ -1058,7 +1058,7 @@
         <v>4</v>
       </c>
       <c r="C45" t="n">
-        <v>126360.9773063609</v>
+        <v>126361.375253529</v>
       </c>
       <c r="D45" t="n">
         <v>0.03269966670781388</v>
@@ -1072,10 +1072,10 @@
         <v>1</v>
       </c>
       <c r="C46" t="n">
-        <v>125997.4955</v>
+        <v>126107.9971</v>
       </c>
       <c r="D46" t="n">
-        <v>-0.002876535257238633</v>
+        <v>-0.002005186735429487</v>
       </c>
     </row>
     <row r="47">
@@ -1086,10 +1086,10 @@
         <v>2</v>
       </c>
       <c r="C47" t="n">
-        <v>129111.1804</v>
+        <v>129054.9995</v>
       </c>
       <c r="D47" t="n">
-        <v>0.02471227612615512</v>
+        <v>0.02336887800749965</v>
       </c>
     </row>
     <row r="48">
@@ -1100,10 +1100,10 @@
         <v>3</v>
       </c>
       <c r="C48" t="n">
-        <v>128696.2283</v>
+        <v>128686.1731</v>
       </c>
       <c r="D48" t="n">
-        <v>-0.003213912991225309</v>
+        <v>-0.002857900906039768</v>
       </c>
     </row>
     <row r="49">
@@ -1114,10 +1114,10 @@
         <v>4</v>
       </c>
       <c r="C49" t="n">
-        <v>131048.0958</v>
+        <v>131003.8303</v>
       </c>
       <c r="D49" t="n">
-        <v>0.01827456430593766</v>
+        <v>0.01801014937478151</v>
       </c>
     </row>
     <row r="50">
@@ -1128,10 +1128,10 @@
         <v>1</v>
       </c>
       <c r="C50" t="n">
-        <v>134111.6696</v>
+        <v>134233.0909</v>
       </c>
       <c r="D50" t="n">
-        <v>0.0233774766531174</v>
+        <v>0.02465012353154084</v>
       </c>
     </row>
     <row r="51">
@@ -1142,10 +1142,10 @@
         <v>2</v>
       </c>
       <c r="C51" t="n">
-        <v>135947.4433</v>
+        <v>135893.7439</v>
       </c>
       <c r="D51" t="n">
-        <v>0.01368839643466813</v>
+        <v>0.01237141295686262</v>
       </c>
     </row>
     <row r="52">
@@ -1156,10 +1156,10 @@
         <v>3</v>
       </c>
       <c r="C52" t="n">
-        <v>138590.7887</v>
+        <v>138577.3806</v>
       </c>
       <c r="D52" t="n">
-        <v>0.0194438772501726</v>
+        <v>0.01974805184538009</v>
       </c>
     </row>
     <row r="53">
@@ -1170,10 +1170,10 @@
         <v>4</v>
       </c>
       <c r="C53" t="n">
-        <v>140785.0983</v>
+        <v>140730.7847</v>
       </c>
       <c r="D53" t="n">
-        <v>0.01583301185153019</v>
+        <v>0.01553936212877138</v>
       </c>
     </row>
     <row r="54">
@@ -1184,10 +1184,10 @@
         <v>1</v>
       </c>
       <c r="C54" t="n">
-        <v>143227.8113</v>
+        <v>143317.9731</v>
       </c>
       <c r="D54" t="n">
-        <v>0.01735065024278915</v>
+        <v>0.01838395490734457</v>
       </c>
     </row>
     <row r="55">
@@ -1198,10 +1198,10 @@
         <v>2</v>
       </c>
       <c r="C55" t="n">
-        <v>145127.5639</v>
+        <v>145054.4202</v>
       </c>
       <c r="D55" t="n">
-        <v>0.01326385275846209</v>
+        <v>0.01211604561828672</v>
       </c>
     </row>
     <row r="56">
@@ -1212,10 +1212,10 @@
         <v>3</v>
       </c>
       <c r="C56" t="n">
-        <v>148141.4186</v>
+        <v>148122.5226</v>
       </c>
       <c r="D56" t="n">
-        <v>0.02076693509495331</v>
+        <v>0.02115138853245369</v>
       </c>
     </row>
     <row r="57">
@@ -1226,10 +1226,10 @@
         <v>4</v>
       </c>
       <c r="C57" t="n">
-        <v>149960.2061</v>
+        <v>149962.0842</v>
       </c>
       <c r="D57" t="n">
-        <v>0.01227737331793044</v>
+        <v>0.01241918897754446</v>
       </c>
     </row>
     <row r="58">
@@ -1240,10 +1240,10 @@
         <v>1</v>
       </c>
       <c r="C58" t="n">
-        <v>150594.8869</v>
+        <v>150365.7438</v>
       </c>
       <c r="D58" t="n">
-        <v>0.00423232813895158</v>
+        <v>0.002691744397614659</v>
       </c>
     </row>
     <row r="59">
@@ -1254,10 +1254,10 @@
         <v>2</v>
       </c>
       <c r="C59" t="n">
-        <v>151691.3942</v>
+        <v>151769.5687</v>
       </c>
       <c r="D59" t="n">
-        <v>0.007281172173714712</v>
+        <v>0.009336068605275027</v>
       </c>
     </row>
     <row r="60">
@@ -1268,10 +1268,10 @@
         <v>3</v>
       </c>
       <c r="C60" t="n">
-        <v>153001.155</v>
+        <v>153090.7174</v>
       </c>
       <c r="D60" t="n">
-        <v>0.00863437775694198</v>
+        <v>0.008704964449174124</v>
       </c>
     </row>
     <row r="61">
@@ -1282,10 +1282,10 @@
         <v>4</v>
       </c>
       <c r="C61" t="n">
-        <v>150425.5639</v>
+        <v>150486.9701</v>
       </c>
       <c r="D61" t="n">
-        <v>-0.01683380167947091</v>
+        <v>-0.01700787183064034</v>
       </c>
     </row>
     <row r="62">
@@ -1296,10 +1296,10 @@
         <v>1</v>
       </c>
       <c r="C62" t="n">
-        <v>150827.7756</v>
+        <v>150954.6375</v>
       </c>
       <c r="D62" t="n">
-        <v>0.002673825442777611</v>
+        <v>0.003107693640779896</v>
       </c>
     </row>
     <row r="63">
@@ -1310,10 +1310,10 @@
         <v>2</v>
       </c>
       <c r="C63" t="n">
-        <v>152493.2533</v>
+        <v>152459.0529</v>
       </c>
       <c r="D63" t="n">
-        <v>0.01104224797703646</v>
+        <v>0.009966009821990474</v>
       </c>
     </row>
     <row r="64">
@@ -1324,10 +1324,10 @@
         <v>3</v>
       </c>
       <c r="C64" t="n">
-        <v>154049.9587</v>
+        <v>153996.6863</v>
       </c>
       <c r="D64" t="n">
-        <v>0.01020835588665325</v>
+        <v>0.01008554999360078</v>
       </c>
     </row>
     <row r="65">
@@ -1338,10 +1338,10 @@
         <v>4</v>
       </c>
       <c r="C65" t="n">
-        <v>155245.0124</v>
+        <v>155205.6233</v>
       </c>
       <c r="D65" t="n">
-        <v>0.00775757234915786</v>
+        <v>0.007850409181174633</v>
       </c>
     </row>
     <row r="66">
@@ -1352,10 +1352,10 @@
         <v>1</v>
       </c>
       <c r="C66" t="n">
-        <v>156686.9061</v>
+        <v>156768.5779</v>
       </c>
       <c r="D66" t="n">
-        <v>0.009287858448455921</v>
+        <v>0.01007021889264248</v>
       </c>
     </row>
     <row r="67">
@@ -1366,10 +1366,10 @@
         <v>2</v>
       </c>
       <c r="C67" t="n">
-        <v>159244.8765</v>
+        <v>159215.0403</v>
       </c>
       <c r="D67" t="n">
-        <v>0.01632536159956777</v>
+        <v>0.01560556606924468</v>
       </c>
     </row>
     <row r="68">
@@ -1380,10 +1380,10 @@
         <v>3</v>
       </c>
       <c r="C68" t="n">
-        <v>160424.5984</v>
+        <v>160387.8128</v>
       </c>
       <c r="D68" t="n">
-        <v>0.007408225155677073</v>
+        <v>0.007365965538118857</v>
       </c>
     </row>
     <row r="69">
@@ -1394,10 +1394,10 @@
         <v>4</v>
       </c>
       <c r="C69" t="n">
-        <v>163794.619</v>
+        <v>163779.569</v>
       </c>
       <c r="D69" t="n">
-        <v>0.02100688194710187</v>
+        <v>0.02114721898620453</v>
       </c>
     </row>
     <row r="70">
@@ -1408,10 +1408,10 @@
         <v>1</v>
       </c>
       <c r="C70" t="n">
-        <v>167223.0681</v>
+        <v>167286.916</v>
       </c>
       <c r="D70" t="n">
-        <v>0.02093139030409774</v>
+        <v>0.02141504597560639</v>
       </c>
     </row>
     <row r="71">
@@ -1422,10 +1422,10 @@
         <v>2</v>
       </c>
       <c r="C71" t="n">
-        <v>169810.3032</v>
+        <v>169747.0668</v>
       </c>
       <c r="D71" t="n">
-        <v>0.01547175954487812</v>
+        <v>0.01470617582549005</v>
       </c>
     </row>
     <row r="72">
@@ -1436,10 +1436,10 @@
         <v>3</v>
       </c>
       <c r="C72" t="n">
-        <v>173255.1511</v>
+        <v>173210.156</v>
       </c>
       <c r="D72" t="n">
-        <v>0.0202864480840288</v>
+        <v>0.02040146710800173</v>
       </c>
     </row>
     <row r="73">
@@ -1450,10 +1450,10 @@
         <v>4</v>
       </c>
       <c r="C73" t="n">
-        <v>174339.4776</v>
+        <v>174383.8611</v>
       </c>
       <c r="D73" t="n">
-        <v>0.006258552736329248</v>
+        <v>0.006776190998869724</v>
       </c>
     </row>
     <row r="74">
@@ -1464,10 +1464,10 @@
         <v>1</v>
       </c>
       <c r="C74" t="n">
-        <v>177267.9611</v>
+        <v>176970.8435</v>
       </c>
       <c r="D74" t="n">
-        <v>0.01679759249204027</v>
+        <v>0.0148349875021776</v>
       </c>
     </row>
     <row r="75">
@@ -1478,10 +1478,10 @@
         <v>2</v>
       </c>
       <c r="C75" t="n">
-        <v>177875.4556</v>
+        <v>177978.8285</v>
       </c>
       <c r="D75" t="n">
-        <v>0.003426984189530469</v>
+        <v>0.005695768749613306</v>
       </c>
     </row>
     <row r="76">
@@ -1492,10 +1492,10 @@
         <v>3</v>
       </c>
       <c r="C76" t="n">
-        <v>177019.5441</v>
+        <v>177110.3455</v>
       </c>
       <c r="D76" t="n">
-        <v>-0.004811858370863287</v>
+        <v>-0.004879698373787211</v>
       </c>
     </row>
     <row r="77">
@@ -1506,10 +1506,10 @@
         <v>4</v>
       </c>
       <c r="C77" t="n">
-        <v>179252.0392</v>
+        <v>179354.9826</v>
       </c>
       <c r="D77" t="n">
-        <v>0.01261157411375358</v>
+        <v>0.01267366450933838</v>
       </c>
     </row>
     <row r="78">
@@ -1520,10 +1520,10 @@
         <v>1</v>
       </c>
       <c r="C78" t="n">
-        <v>181471.8698</v>
+        <v>181618.7873</v>
       </c>
       <c r="D78" t="n">
-        <v>0.01238385130739417</v>
+        <v>0.01262192255371453</v>
       </c>
     </row>
     <row r="79">
@@ -1534,10 +1534,10 @@
         <v>2</v>
       </c>
       <c r="C79" t="n">
-        <v>187576.3127</v>
+        <v>187529.4877</v>
       </c>
       <c r="D79" t="n">
-        <v>0.03363850775730537</v>
+        <v>0.03254454281889152</v>
       </c>
     </row>
     <row r="80">
@@ -1548,10 +1548,10 @@
         <v>3</v>
       </c>
       <c r="C80" t="n">
-        <v>188086.5846</v>
+        <v>188017.7345</v>
       </c>
       <c r="D80" t="n">
-        <v>0.002720342950850663</v>
+        <v>0.002603573475234322</v>
       </c>
     </row>
     <row r="81">
@@ -1562,10 +1562,10 @@
         <v>4</v>
       </c>
       <c r="C81" t="n">
-        <v>190804.2329</v>
+        <v>190772.9905</v>
       </c>
       <c r="D81" t="n">
-        <v>0.01444892152079613</v>
+        <v>0.01465423465146598</v>
       </c>
     </row>
     <row r="82">
@@ -1576,10 +1576,10 @@
         <v>1</v>
       </c>
       <c r="C82" t="n">
-        <v>193552.9298</v>
+        <v>193660.5985</v>
       </c>
       <c r="D82" t="n">
-        <v>0.01440584864509065</v>
+        <v>0.015136356527367</v>
       </c>
     </row>
     <row r="83">
@@ -1590,10 +1590,10 @@
         <v>2</v>
       </c>
       <c r="C83" t="n">
-        <v>194035.6944</v>
+        <v>193990.1918</v>
       </c>
       <c r="D83" t="n">
-        <v>0.002494225225620816</v>
+        <v>0.001701912017998852</v>
       </c>
     </row>
     <row r="84">
@@ -1604,10 +1604,10 @@
         <v>3</v>
       </c>
       <c r="C84" t="n">
-        <v>195997.7779</v>
+        <v>195956.5612</v>
       </c>
       <c r="D84" t="n">
-        <v>0.01011197195478464</v>
+        <v>0.01013643721754387</v>
       </c>
     </row>
     <row r="85">
@@ -1618,10 +1618,10 @@
         <v>4</v>
       </c>
       <c r="C85" t="n">
-        <v>198002.5978</v>
+        <v>197981.6485</v>
       </c>
       <c r="D85" t="n">
-        <v>0.01022878892546863</v>
+        <v>0.01033436843144608</v>
       </c>
     </row>
     <row r="86">
@@ -1632,10 +1632,10 @@
         <v>1</v>
       </c>
       <c r="C86" t="n">
-        <v>199174.7801</v>
+        <v>199260.6494</v>
       </c>
       <c r="D86" t="n">
-        <v>0.00592003495420812</v>
+        <v>0.006460199264377797</v>
       </c>
     </row>
     <row r="87">
@@ -1646,10 +1646,10 @@
         <v>2</v>
       </c>
       <c r="C87" t="n">
-        <v>200715.0508</v>
+        <v>200645.7306</v>
       </c>
       <c r="D87" t="n">
-        <v>0.007733261707263628</v>
+        <v>0.006951102509053619</v>
       </c>
     </row>
     <row r="88">
@@ -1660,10 +1660,10 @@
         <v>3</v>
       </c>
       <c r="C88" t="n">
-        <v>202719.1143</v>
+        <v>202671.6638</v>
       </c>
       <c r="D88" t="n">
-        <v>0.00998461994759392</v>
+        <v>0.01009706607731831</v>
       </c>
     </row>
     <row r="89">
@@ -1674,10 +1674,10 @@
         <v>4</v>
       </c>
       <c r="C89" t="n">
-        <v>202083.0548</v>
+        <v>202113.9562</v>
       </c>
       <c r="D89" t="n">
-        <v>-0.003137639497865385</v>
+        <v>-0.00275177886016853</v>
       </c>
     </row>
     <row r="90">
@@ -1688,10 +1688,10 @@
         <v>1</v>
       </c>
       <c r="C90" t="n">
-        <v>204161.2218</v>
+        <v>203832.3291</v>
       </c>
       <c r="D90" t="n">
-        <v>0.01028372716384718</v>
+        <v>0.008502000219616779</v>
       </c>
     </row>
     <row r="91">
@@ -1702,10 +1702,10 @@
         <v>2</v>
       </c>
       <c r="C91" t="n">
-        <v>204974.5016</v>
+        <v>205120.1897</v>
       </c>
       <c r="D91" t="n">
-        <v>0.003983517500677491</v>
+        <v>0.006318235216594026</v>
       </c>
     </row>
     <row r="92">
@@ -1716,10 +1716,10 @@
         <v>3</v>
       </c>
       <c r="C92" t="n">
-        <v>205519.2187</v>
+        <v>205623.0613</v>
       </c>
       <c r="D92" t="n">
-        <v>0.002657487130096836</v>
+        <v>0.002451594846589744</v>
       </c>
     </row>
     <row r="93">
@@ -1730,10 +1730,10 @@
         <v>4</v>
       </c>
       <c r="C93" t="n">
-        <v>206834.0579</v>
+        <v>206913.4199</v>
       </c>
       <c r="D93" t="n">
-        <v>0.0063976459638031</v>
+        <v>0.00627535934851875</v>
       </c>
     </row>
     <row r="94">
@@ -1744,10 +1744,10 @@
         <v>1</v>
       </c>
       <c r="C94" t="n">
-        <v>206566.6775</v>
+        <v>206757.2117</v>
       </c>
       <c r="D94" t="n">
-        <v>-0.001292729073319676</v>
+        <v>-0.0007549447497193773</v>
       </c>
     </row>
     <row r="95">
@@ -1758,10 +1758,10 @@
         <v>2</v>
       </c>
       <c r="C95" t="n">
-        <v>207530.0582</v>
+        <v>207539.18</v>
       </c>
       <c r="D95" t="n">
-        <v>0.004663775937433057</v>
+        <v>0.00378206057999364</v>
       </c>
     </row>
     <row r="96">
@@ -1772,10 +1772,10 @@
         <v>3</v>
       </c>
       <c r="C96" t="n">
-        <v>208795.5456</v>
+        <v>208682.8678</v>
       </c>
       <c r="D96" t="n">
-        <v>0.006097851130463461</v>
+        <v>0.005510707905851842</v>
       </c>
     </row>
     <row r="97">
@@ -1786,10 +1786,10 @@
         <v>4</v>
       </c>
       <c r="C97" t="n">
-        <v>209763.7187</v>
+        <v>209676.7405</v>
       </c>
       <c r="D97" t="n">
-        <v>0.004636943270115435</v>
+        <v>0.004762598436937937</v>
       </c>
     </row>
     <row r="98">
@@ -1800,10 +1800,10 @@
         <v>1</v>
       </c>
       <c r="C98" t="n">
-        <v>210237.9595</v>
+        <v>210404.0478</v>
       </c>
       <c r="D98" t="n">
-        <v>0.002260833298241893</v>
+        <v>0.003468707584187047</v>
       </c>
     </row>
     <row r="99">
@@ -1814,10 +1814,10 @@
         <v>2</v>
       </c>
       <c r="C99" t="n">
-        <v>213136.6749</v>
+        <v>213221.7791</v>
       </c>
       <c r="D99" t="n">
-        <v>0.01378778317147811</v>
+        <v>0.01339200138715202</v>
       </c>
     </row>
     <row r="100">
@@ -1828,10 +1828,10 @@
         <v>3</v>
       </c>
       <c r="C100" t="n">
-        <v>214679.7169</v>
+        <v>214537.2762</v>
       </c>
       <c r="D100" t="n">
-        <v>0.007239683178523526</v>
+        <v>0.006169618814516165</v>
       </c>
     </row>
     <row r="101">
@@ -1842,10 +1842,10 @@
         <v>4</v>
       </c>
       <c r="C101" t="n">
-        <v>215953.6487</v>
+        <v>215844.8969</v>
       </c>
       <c r="D101" t="n">
-        <v>0.005934104154764697</v>
+        <v>0.006095074586390137</v>
       </c>
     </row>
     <row r="102">
@@ -1856,10 +1856,10 @@
         <v>1</v>
       </c>
       <c r="C102" t="n">
-        <v>217669.2957</v>
+        <v>217897.1681</v>
       </c>
       <c r="D102" t="n">
-        <v>0.007944514993508456</v>
+        <v>0.009508083023852087</v>
       </c>
     </row>
     <row r="103">
@@ -1870,10 +1870,10 @@
         <v>2</v>
       </c>
       <c r="C103" t="n">
-        <v>219578.7339</v>
+        <v>219673.4809</v>
       </c>
       <c r="D103" t="n">
-        <v>0.008772198181923097</v>
+        <v>0.008152069232881365</v>
       </c>
     </row>
     <row r="104">
@@ -1884,10 +1884,10 @@
         <v>3</v>
       </c>
       <c r="C104" t="n">
-        <v>221312.4139</v>
+        <v>221065.7358</v>
       </c>
       <c r="D104" t="n">
-        <v>0.007895482268285514</v>
+        <v>0.006337837841399629</v>
       </c>
     </row>
     <row r="105">
@@ -1898,10 +1898,10 @@
         <v>4</v>
       </c>
       <c r="C105" t="n">
-        <v>222663.5565</v>
+        <v>222587.6152</v>
       </c>
       <c r="D105" t="n">
-        <v>0.006105136969905889</v>
+        <v>0.006884284416545094</v>
       </c>
     </row>
     <row r="106">
@@ -1912,10 +1912,10 @@
         <v>1</v>
       </c>
       <c r="C106" t="n">
-        <v>218395.0084</v>
+        <v>218242.0591</v>
       </c>
       <c r="D106" t="n">
-        <v>-0.0191703939661092</v>
+        <v>-0.01952290155988867</v>
       </c>
     </row>
     <row r="107">
@@ -1926,10 +1926,10 @@
         <v>2</v>
       </c>
       <c r="C107" t="n">
-        <v>182829.6348</v>
+        <v>183134.6644</v>
       </c>
       <c r="D107" t="n">
-        <v>-0.1628488391770404</v>
+        <v>-0.1608644770159245</v>
       </c>
     </row>
     <row r="108">
@@ -1940,10 +1940,10 @@
         <v>3</v>
       </c>
       <c r="C108" t="n">
-        <v>201256.4906</v>
+        <v>201141.6042</v>
       </c>
       <c r="D108" t="n">
-        <v>0.1007870295215401</v>
+        <v>0.09832622272247438</v>
       </c>
     </row>
     <row r="109">
@@ -1954,10 +1954,10 @@
         <v>4</v>
       </c>
       <c r="C109" t="n">
-        <v>215418.8662</v>
+        <v>215381.6723</v>
       </c>
       <c r="D109" t="n">
-        <v>0.07036978314477271</v>
+        <v>0.07079623410898495</v>
       </c>
     </row>
     <row r="110">
@@ -1968,10 +1968,10 @@
         <v>1</v>
       </c>
       <c r="C110" t="n">
-        <v>221803.8831</v>
+        <v>222283.7627</v>
       </c>
       <c r="D110" t="n">
-        <v>0.02964000791867516</v>
+        <v>0.03204585759918444</v>
       </c>
     </row>
     <row r="111">
@@ -1982,10 +1982,10 @@
         <v>2</v>
       </c>
       <c r="C111" t="n">
-        <v>216740.0427</v>
+        <v>216884.6998</v>
       </c>
       <c r="D111" t="n">
-        <v>-0.0228302603598558</v>
+        <v>-0.02428905662932612</v>
       </c>
     </row>
     <row r="112">
@@ -1996,10 +1996,10 @@
         <v>3</v>
       </c>
       <c r="C112" t="n">
-        <v>228413.187</v>
+        <v>228045.5012</v>
       </c>
       <c r="D112" t="n">
-        <v>0.05385781120361477</v>
+        <v>0.05145960692613127</v>
       </c>
     </row>
     <row r="113">
@@ -2010,10 +2010,10 @@
         <v>4</v>
       </c>
       <c r="C113" t="n">
-        <v>239285.8872</v>
+        <v>239029.0362</v>
       </c>
       <c r="D113" t="n">
-        <v>0.04760101788694016</v>
+        <v>0.0481637872363343</v>
       </c>
     </row>
     <row r="114">
@@ -2024,10 +2024,10 @@
         <v>1</v>
       </c>
       <c r="C114" t="n">
-        <v>239550.0983</v>
+        <v>240009.7479</v>
       </c>
       <c r="D114" t="n">
-        <v>0.001104164993145584</v>
+        <v>0.004102897771714353</v>
       </c>
     </row>
     <row r="115">
@@ -2038,10 +2038,10 @@
         <v>2</v>
       </c>
       <c r="C115" t="n">
-        <v>243436.201</v>
+        <v>243631.2471</v>
       </c>
       <c r="D115" t="n">
-        <v>0.01622250513599566</v>
+        <v>0.01508896714273833</v>
       </c>
     </row>
     <row r="116">
@@ -2052,10 +2052,10 @@
         <v>3</v>
       </c>
       <c r="C116" t="n">
-        <v>245182.7627</v>
+        <v>244793.934</v>
       </c>
       <c r="D116" t="n">
-        <v>0.007174617796471328</v>
+        <v>0.00477232257290372</v>
       </c>
     </row>
     <row r="117">
@@ -2066,10 +2066,10 @@
         <v>4</v>
       </c>
       <c r="C117" t="n">
-        <v>244485.9381</v>
+        <v>244220.071</v>
       </c>
       <c r="D117" t="n">
-        <v>-0.002842061947285424</v>
+        <v>-0.002344269690931156</v>
       </c>
     </row>
     <row r="118">
@@ -2080,10 +2080,10 @@
         <v>1</v>
       </c>
       <c r="C118" t="n">
-        <v>246017.7267</v>
+        <v>246512.5278</v>
       </c>
       <c r="D118" t="n">
-        <v>0.006265344387101246</v>
+        <v>0.00938684847077953</v>
       </c>
     </row>
     <row r="119">
@@ -2094,10 +2094,10 @@
         <v>2</v>
       </c>
       <c r="C119" t="n">
-        <v>244468.8669</v>
+        <v>244647.3407</v>
       </c>
       <c r="D119" t="n">
-        <v>-0.006295724380417256</v>
+        <v>-0.007566297407461842</v>
       </c>
     </row>
     <row r="120">
@@ -2108,10 +2108,10 @@
         <v>3</v>
       </c>
       <c r="C120" t="n">
-        <v>244178.5966</v>
+        <v>243822.3181</v>
       </c>
       <c r="D120" t="n">
-        <v>-0.00118735078082044</v>
+        <v>-0.003372293349436783</v>
       </c>
     </row>
     <row r="121">
@@ -2122,10 +2122,10 @@
         <v>4</v>
       </c>
       <c r="C121" t="n">
-        <v>246177.8098</v>
+        <v>245860.8135</v>
       </c>
       <c r="D121" t="n">
-        <v>0.008187503851023514</v>
+        <v>0.00836057755452857</v>
       </c>
     </row>
     <row r="122">
@@ -2136,10 +2136,10 @@
         <v>1</v>
       </c>
       <c r="C122" t="n">
-        <v>246721.9338</v>
+        <v>246462.7026</v>
       </c>
       <c r="D122" t="n">
-        <v>0.002210288573296193</v>
+        <v>0.002448088784185121</v>
       </c>
     </row>
     <row r="123">
@@ -2150,10 +2150,10 @@
         <v>2</v>
       </c>
       <c r="C123" t="n">
-        <v>248617.8079</v>
+        <v>248813.1198</v>
       </c>
       <c r="D123" t="n">
-        <v>0.007684254378197641</v>
+        <v>0.0095366040183964</v>
       </c>
     </row>
     <row r="124">
@@ -2164,10 +2164,10 @@
         <v>3</v>
       </c>
       <c r="C124" t="n">
-        <v>248237.3609</v>
+        <v>248008.9379</v>
       </c>
       <c r="D124" t="n">
-        <v>-0.001530248388937006</v>
+        <v>-0.003232071928708669</v>
       </c>
     </row>
     <row r="125">
@@ -2178,10 +2178,10 @@
         <v>4</v>
       </c>
       <c r="C125" t="n">
-        <v>251912.8973</v>
+        <v>252205.2397</v>
       </c>
       <c r="D125" t="n">
-        <v>0.01480653994497083</v>
+        <v>0.01691996198012835</v>
       </c>
     </row>
     <row r="126">
@@ -2192,10 +2192,10 @@
         <v>1</v>
       </c>
       <c r="C126" t="n">
-        <v>253089.4119</v>
+        <v>253276.2598</v>
       </c>
       <c r="D126" t="n">
-        <v>0.00467032300691983</v>
+        <v>0.004246621129973205</v>
       </c>
     </row>
     <row r="127">
@@ -2206,10 +2206,10 @@
         <v>2</v>
       </c>
       <c r="C127" t="n">
-        <v>253990.2704</v>
+        <v>253364.3977</v>
       </c>
       <c r="D127" t="n">
-        <v>0.003559447600897547</v>
+        <v>0.0003479911621784293</v>
       </c>
     </row>
     <row r="128">
@@ -2220,10 +2220,10 @@
         <v>3</v>
       </c>
       <c r="C128" t="n">
-        <v>257201.0399</v>
+        <v>257168.6847</v>
       </c>
       <c r="D128" t="n">
-        <v>0.01264130903496219</v>
+        <v>0.01501508118162898</v>
       </c>
     </row>
     <row r="129">
@@ -2234,10 +2234,24 @@
         <v>4</v>
       </c>
       <c r="C129" t="n">
-        <v>257510.2116</v>
+        <v>257263.5814</v>
       </c>
       <c r="D129" t="n">
-        <v>0.001202062402703374</v>
+        <v>0.000369005659109245</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B130" t="n">
+        <v>1</v>
+      </c>
+      <c r="C130" t="n">
+        <v>258780.6605</v>
+      </c>
+      <c r="D130" t="n">
+        <v>0.005896983520730759</v>
       </c>
     </row>
   </sheetData>

</xml_diff>